<commit_message>
updated CV and added to companies xcel and presentation
</commit_message>
<xml_diff>
--- a/research/Companies by size.xlsx
+++ b/research/Companies by size.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Bubbles\Documents\GitHub\Applied-Software-Project-Management_CA\research\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2ED8CAF-5357-4C59-AD74-192F571E16CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDC92492-3095-4FF1-A60A-C03B92D964A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{CD4061D8-C85C-4E4F-A74B-9467D67D851A}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="8">
   <si>
     <t>Multinational</t>
   </si>
@@ -48,6 +48,18 @@
   </si>
   <si>
     <t>Location</t>
+  </si>
+  <si>
+    <t>IBM</t>
+  </si>
+  <si>
+    <t>Charlemont Exchange, WeWork Office Space, Temple Bar, Dublin</t>
+  </si>
+  <si>
+    <t>Amazon</t>
+  </si>
+  <si>
+    <t>Burlington Rd, Dublin 4, D04 HH21</t>
   </si>
 </sst>
 </file>
@@ -419,11 +431,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A979AC8B-B2DA-4541-8D88-56D3AC78779A}">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.85546875" customWidth="1"/>
-    <col min="2" max="2" width="33.140625" customWidth="1"/>
+    <col min="2" max="2" width="61" customWidth="1"/>
     <col min="3" max="3" width="25.7109375" customWidth="1"/>
     <col min="4" max="4" width="32.7109375" customWidth="1"/>
     <col min="5" max="5" width="26.85546875" customWidth="1"/>
@@ -448,6 +460,22 @@
       </c>
       <c r="F1" t="s">
         <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
more work on Xcel sheet
</commit_message>
<xml_diff>
--- a/research/Companies by size.xlsx
+++ b/research/Companies by size.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Bubbles\Documents\GitHub\Applied-Software-Project-Management_CA\research\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDC92492-3095-4FF1-A60A-C03B92D964A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1D0C5CB-AF07-4005-8F95-DA3DB35F6484}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{CD4061D8-C85C-4E4F-A74B-9467D67D851A}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="10">
   <si>
     <t>Multinational</t>
   </si>
@@ -60,6 +60,12 @@
   </si>
   <si>
     <t>Burlington Rd, Dublin 4, D04 HH21</t>
+  </si>
+  <si>
+    <t>Prometric</t>
+  </si>
+  <si>
+    <t>Dundalk</t>
   </si>
 </sst>
 </file>
@@ -431,7 +437,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A979AC8B-B2DA-4541-8D88-56D3AC78779A}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.85546875" customWidth="1"/>
@@ -476,6 +482,14 @@
       </c>
       <c r="B3" t="s">
         <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added more companies to excel sheet
</commit_message>
<xml_diff>
--- a/research/Companies by size.xlsx
+++ b/research/Companies by size.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Bubbles\Documents\GitHub\Applied-Software-Project-Management_CA\research\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matth\OneDrive\Documents\GitHub\Applied-Software-Project-Management_CA\research\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1D0C5CB-AF07-4005-8F95-DA3DB35F6484}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4D56FBC-1BD4-45DA-BA5D-6CA365BA324A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{CD4061D8-C85C-4E4F-A74B-9467D67D851A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{CD4061D8-C85C-4E4F-A74B-9467D67D851A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="14">
   <si>
     <t>Multinational</t>
   </si>
@@ -66,6 +66,18 @@
   </si>
   <si>
     <t>Dundalk</t>
+  </si>
+  <si>
+    <t>Riot Games</t>
+  </si>
+  <si>
+    <t>The Observatory Building, 7-11 Sir John Rogerson's Quay</t>
+  </si>
+  <si>
+    <t>DIGIT, a Scopely Studio</t>
+  </si>
+  <si>
+    <t>4 Prince's Street South, Dublin, Dublin 2 IE</t>
   </si>
 </sst>
 </file>
@@ -437,18 +449,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A979AC8B-B2DA-4541-8D88-56D3AC78779A}">
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.85546875" customWidth="1"/>
+    <col min="1" max="1" width="20.88671875" customWidth="1"/>
     <col min="2" max="2" width="61" customWidth="1"/>
-    <col min="3" max="3" width="25.7109375" customWidth="1"/>
-    <col min="4" max="4" width="32.7109375" customWidth="1"/>
-    <col min="5" max="5" width="26.85546875" customWidth="1"/>
-    <col min="6" max="6" width="32.28515625" customWidth="1"/>
+    <col min="3" max="3" width="25.6640625" customWidth="1"/>
+    <col min="4" max="4" width="39.33203125" customWidth="1"/>
+    <col min="5" max="5" width="26.88671875" customWidth="1"/>
+    <col min="6" max="6" width="32.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -468,15 +480,21 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
       <c r="B2" t="s">
         <v>5</v>
       </c>
+      <c r="C2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -484,12 +502,20 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
       <c r="B4" t="s">
         <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -498,15 +524,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008C4A6D6B560E8246B29703C8C6568C34" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="69f712a45ceab6f59ecd8b3843db96e2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="ceb90afc-e9ec-43ec-aa13-f18c9abd74cb" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="bbc2f7de990a4bff2ccc684cc776d44e" ns3:_="">
     <xsd:import namespace="ceb90afc-e9ec-43ec-aa13-f18c9abd74cb"/>
@@ -686,6 +703,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -695,14 +721,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6FAE861A-34C6-45DB-A0AC-C2E6F2A76013}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4334100B-E50D-4DFC-845F-45E0E36A7578}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -720,6 +738,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6FAE861A-34C6-45DB-A0AC-C2E6F2A76013}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{544E77EA-B497-4006-B187-65730B7F9E4C}">
   <ds:schemaRefs>

</xml_diff>